<commit_message>
Correct review status labels
</commit_message>
<xml_diff>
--- a/Downloads/pkrishnakishore-Cochrane-2d9e7d5/pkrishnakishore-Cochrane-2d9e7d5/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
+++ b/Downloads/pkrishnakishore-Cochrane-2d9e7d5/pkrishnakishore-Cochrane-2d9e7d5/AI-Platform-Study/dashboard/cochrane_dashboard_backend_template.xlsx
@@ -2400,7 +2400,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>AI-assisted abstract screening complete</t>
+          <t>Abstract Screening</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -36388,7 +36388,7 @@
       </c>
       <c r="B10" s="9" t="inlineStr">
         <is>
-          <t>Updated 2026-07-30: Fruit &amp; Vegetable AI abstract screening complete; conventional consolidation and full-text setup pending.</t>
+          <t>Updated 2026-07-30: Corrected review status labels: Psoriasis and Fruit &amp; Vegetable in Abstract Screening; Vitamin C in Setup phase.</t>
         </is>
       </c>
     </row>
@@ -36846,7 +36846,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>AI-assisted abstract screening complete</t>
+          <t>Abstract Screening</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">

</xml_diff>